<commit_message>
base case 15 dd
</commit_message>
<xml_diff>
--- a/case_studies/base_case_10_dd/2030/technologies.xlsx
+++ b/case_studies/base_case_10_dd/2030/technologies.xlsx
@@ -682,7 +682,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>0</v>
@@ -694,7 +694,7 @@
         <v>53.53</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>150.56</v>
+        <v>150.75</v>
       </c>
       <c r="K2" s="3" t="n">
         <v>0</v>
@@ -1164,7 +1164,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0</v>
@@ -1261,7 +1261,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
min modifications on case studies
</commit_message>
<xml_diff>
--- a/case_studies/base_case_10_dd/2030/technologies.xlsx
+++ b/case_studies/base_case_10_dd/2030/technologies.xlsx
@@ -682,7 +682,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>0</v>
@@ -694,7 +694,7 @@
         <v>53.53</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>150.75</v>
+        <v>150.99</v>
       </c>
       <c r="K2" s="3" t="n">
         <v>0</v>
@@ -1164,7 +1164,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0</v>
@@ -1203,10 +1203,10 @@
         <v>0</v>
       </c>
       <c r="R7" s="5" t="n">
-        <v>19.82</v>
+        <v>19.57</v>
       </c>
       <c r="S7" s="5" t="n">
-        <v>15.67</v>
+        <v>15.8</v>
       </c>
       <c r="T7" s="5" t="n">
         <v>48.52</v>
@@ -1218,7 +1218,7 @@
         <v>1.43</v>
       </c>
       <c r="W7" s="5" t="n">
-        <v>19.43</v>
+        <v>19.18</v>
       </c>
       <c r="X7" s="5" t="n">
         <v>0</v>
@@ -1261,7 +1261,7 @@
         <v>0</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>0</v>
@@ -1273,10 +1273,10 @@
         <v>0</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>65.55</v>
+        <v>65.58</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>160.77</v>
+        <v>161.65</v>
       </c>
       <c r="K8" s="3" t="n">
         <v>0</v>
@@ -1294,16 +1294,16 @@
         <v>0</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>165.93</v>
+        <v>165.99</v>
       </c>
       <c r="Q8" s="3" t="n">
-        <v>219.24</v>
+        <v>219.11</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>45.07</v>
+        <v>45.09</v>
       </c>
       <c r="S8" s="3" t="n">
-        <v>36.27</v>
+        <v>36.14</v>
       </c>
       <c r="T8" s="3" t="n">
         <v>110.4</v>
@@ -1315,7 +1315,7 @@
         <v>0</v>
       </c>
       <c r="W8" s="3" t="n">
-        <v>45.07</v>
+        <v>45.09</v>
       </c>
       <c r="X8" s="3" t="n">
         <v>0</v>

</xml_diff>